<commit_message>
Final forced template sync with premium version
</commit_message>
<xml_diff>
--- a/Nifty50.xlsx
+++ b/Nifty50.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/04e84142cbb0cbb1/Documents/tradin/tem/108TS/108TS_Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="8_{0BBEC706-7F80-4AFF-A4CB-44519049E019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7ECF8711-B09F-44CE-8108-77550AE74D61}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="8_{0BBEC706-7F80-4AFF-A4CB-44519049E019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82085A29-ABBF-4DB1-BF98-19C68AADA277}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -858,76 +858,6 @@
   <dxfs count="42">
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -978,6 +908,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1008,11 +948,41 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1088,21 +1058,31 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1135,6 +1115,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -1160,6 +1150,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1272,21 +1272,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3537,14 +3537,6 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AB23" s="5">
-        <f t="shared" ref="AB23:AB37" si="21">P23-O23</f>
-        <v>0</v>
-      </c>
-      <c r="AC23" s="5">
-        <f t="shared" ref="AC23:AC37" si="22">W23-V23</f>
-        <v>0</v>
-      </c>
       <c r="AD23" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -3632,14 +3624,6 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AB24" s="5">
-        <f t="shared" si="21"/>
-        <v>0</v>
-      </c>
-      <c r="AC24" s="5">
-        <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
       <c r="AD24" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -3727,14 +3711,6 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AB25" s="5">
-        <f t="shared" si="21"/>
-        <v>0</v>
-      </c>
-      <c r="AC25" s="5">
-        <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
       <c r="AD25" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -3822,14 +3798,6 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AB26" s="5">
-        <f t="shared" si="21"/>
-        <v>0</v>
-      </c>
-      <c r="AC26" s="5">
-        <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
       <c r="AD26" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -3917,14 +3885,6 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AB27" s="5">
-        <f t="shared" si="21"/>
-        <v>0</v>
-      </c>
-      <c r="AC27" s="5">
-        <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
       <c r="AD27" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -4012,14 +3972,6 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
-      <c r="AB28" s="5">
-        <f t="shared" si="21"/>
-        <v>0</v>
-      </c>
-      <c r="AC28" s="5">
-        <f t="shared" si="22"/>
-        <v>0</v>
-      </c>
       <c r="AD28" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -4108,11 +4060,11 @@
         <v>0</v>
       </c>
       <c r="AB29" s="5">
-        <f t="shared" si="21"/>
+        <f t="shared" ref="AB23:AB49" si="21">P29-O29</f>
         <v>0</v>
       </c>
       <c r="AC29" s="5">
-        <f t="shared" si="22"/>
+        <f t="shared" ref="AC23:AC49" si="22">W29-V29</f>
         <v>0</v>
       </c>
       <c r="AD29" s="5">
@@ -4962,6 +4914,14 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
+      <c r="AB38" s="5">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="AC38" s="5">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
       <c r="AD38" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -5049,6 +5009,14 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
+      <c r="AB39" s="5">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="AC39" s="5">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
       <c r="AD39" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -5136,6 +5104,14 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
+      <c r="AB40" s="5">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="AC40" s="5">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
       <c r="AD40" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -5223,6 +5199,14 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
+      <c r="AB41" s="5">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="AC41" s="5">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
       <c r="AD41" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -5310,6 +5294,14 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
+      <c r="AB42" s="5">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="AC42" s="5">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
       <c r="AD42" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -5397,6 +5389,14 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
+      <c r="AB43" s="5">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="AC43" s="5">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
       <c r="AD43" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -5484,6 +5484,14 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
+      <c r="AB44" s="5">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="AC44" s="5">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
       <c r="AD44" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -5571,6 +5579,14 @@
         <f t="shared" si="15"/>
         <v>0</v>
       </c>
+      <c r="AB45" s="5">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="AC45" s="5">
+        <f t="shared" si="22"/>
+        <v>0</v>
+      </c>
       <c r="AD45" s="5">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -5656,6 +5672,14 @@
       </c>
       <c r="AA46" s="4">
         <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="AB46" s="5">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="AC46" s="5">
+        <f t="shared" si="22"/>
         <v>0</v>
       </c>
       <c r="AD46" s="5">
@@ -9185,10 +9209,10 @@
     <mergeCell ref="H78:L78"/>
   </mergeCells>
   <conditionalFormatting sqref="B86">
-    <cfRule type="cellIs" dxfId="41" priority="27" operator="lessThan">
+    <cfRule type="cellIs" dxfId="41" priority="28" operator="greaterThan">
       <formula>$D$58</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="28" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="40" priority="27" operator="lessThan">
       <formula>$D$58</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9209,12 +9233,12 @@
       <formula>NOT(ISERROR(SEARCH("Gap Up ",C86)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F85:H85 F86:V89 F90:G94 K90:V94 F95:V97 F103:V121 K98:V102 F98:G102">
+  <conditionalFormatting sqref="F85:H85 F86:V89 F90:G94 K90:V94 F95:V97 F98:G102 K98:V102 F103:V121">
     <cfRule type="containsText" dxfId="34" priority="60" operator="containsText" text="CE">
       <formula>NOT(ISERROR(SEARCH("CE",F85)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F86:V89 F85:H85 F90:G94 K90:V94 F95:V97 F103:V121 K98:V102 F98:G102">
+  <conditionalFormatting sqref="F86:V89 F85:H85 F90:G94 K90:V94 F95:V97 F98:G102 K98:V102 F103:V121">
     <cfRule type="containsText" dxfId="33" priority="59" operator="containsText" text="PE">
       <formula>NOT(ISERROR(SEARCH("PE",F85)))</formula>
     </cfRule>
@@ -9228,29 +9252,29 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H79:K79">
-    <cfRule type="containsText" dxfId="30" priority="50" operator="containsText" text="CE">
+    <cfRule type="containsText" dxfId="30" priority="49" operator="containsText" text="PE">
+      <formula>NOT(ISERROR(SEARCH("PE",H79)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="29" priority="50" operator="containsText" text="CE">
       <formula>NOT(ISERROR(SEARCH("CE",H79)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="29" priority="49" operator="containsText" text="PE">
-      <formula>NOT(ISERROR(SEARCH("PE",H79)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I80:I85">
-    <cfRule type="cellIs" dxfId="28" priority="45" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="28" priority="44" operator="lessThan">
       <formula>$D$58</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="45" operator="greaterThan">
+      <formula>$D$58</formula>
+    </cfRule>
+    <cfRule type="duplicateValues" dxfId="26" priority="43"/>
+    <cfRule type="cellIs" dxfId="25" priority="46" operator="equal">
       <formula>$A$70</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="47" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="47" operator="greaterThan">
       <formula>24500</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="48" operator="lessThan">
+    <cfRule type="cellIs" dxfId="23" priority="48" operator="lessThan">
       <formula>24500</formula>
-    </cfRule>
-    <cfRule type="duplicateValues" dxfId="24" priority="43"/>
-    <cfRule type="cellIs" dxfId="23" priority="44" operator="lessThan">
-      <formula>$D$58</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I91">
@@ -9268,93 +9292,93 @@
       <formula>$J$93</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I99">
+    <cfRule type="cellIs" dxfId="19" priority="7" operator="greaterThan">
+      <formula>$J$91</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I100">
+    <cfRule type="cellIs" dxfId="18" priority="5" operator="lessThan">
+      <formula>$J$92</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I101">
+    <cfRule type="cellIs" dxfId="17" priority="2" operator="greaterThan">
+      <formula>$J$93</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J91">
-    <cfRule type="cellIs" dxfId="19" priority="10" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="16" priority="10" operator="greaterThan">
       <formula>$I$91</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="13" operator="greaterThan">
       <formula>$I$91</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J92">
-    <cfRule type="cellIs" dxfId="17" priority="11" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="11" operator="lessThan">
       <formula>$I$92</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J93">
-    <cfRule type="cellIs" dxfId="16" priority="8" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="13" priority="8" operator="greaterThan">
+      <formula>$I$93</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J99">
+    <cfRule type="cellIs" dxfId="12" priority="6" operator="greaterThan">
+      <formula>$I$91</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="greaterThan">
+      <formula>$I$91</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J100">
+    <cfRule type="cellIs" dxfId="10" priority="4" operator="lessThan">
+      <formula>$I$92</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J101">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="greaterThan">
       <formula>$I$93</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J80:K85">
-    <cfRule type="cellIs" dxfId="15" priority="51" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="52" operator="greaterThan">
       <formula>$D$79</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="52" operator="greaterThan">
-      <formula>$D$79</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="53" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="53" operator="lessThan">
       <formula>$S$2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="54" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="54" operator="greaterThan">
       <formula>$S$2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="51" operator="lessThan">
+      <formula>$D$79</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L80:L85">
-    <cfRule type="containsText" dxfId="11" priority="17" operator="containsText" text="ITM">
+    <cfRule type="containsText" dxfId="4" priority="17" operator="containsText" text="ITM">
       <formula>NOT(ISERROR(SEARCH("ITM",L80)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="16" operator="containsText" text="OTM">
+    <cfRule type="containsText" dxfId="3" priority="16" operator="containsText" text="OTM">
       <formula>NOT(ISERROR(SEARCH("OTM",L80)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="15" operator="containsText" text="ATM">
+    <cfRule type="containsText" dxfId="2" priority="15" operator="containsText" text="ATM">
       <formula>NOT(ISERROR(SEARCH("ATM",L80)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N85 Q85:V85 O87:P87 E101">
-    <cfRule type="containsText" dxfId="8" priority="57" operator="containsText" text="PE">
+    <cfRule type="containsText" dxfId="1" priority="57" operator="containsText" text="PE">
       <formula>NOT(ISERROR(SEARCH("PE",E85)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="58" operator="containsText" text="CE">
+    <cfRule type="containsText" dxfId="0" priority="58" operator="containsText" text="CE">
       <formula>NOT(ISERROR(SEARCH("CE",E85)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD1:AD1048576">
     <cfRule type="top10" priority="66" bottom="1" rank="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I99">
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="greaterThan">
-      <formula>$J$91</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I100">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="lessThan">
-      <formula>$J$92</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I101">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="greaterThan">
-      <formula>$J$93</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J99">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
-      <formula>$I$91</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="6" operator="greaterThan">
-      <formula>$I$91</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J100">
-    <cfRule type="cellIs" dxfId="1" priority="4" operator="lessThan">
-      <formula>$I$92</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J101">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
-      <formula>$I$93</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>